<commit_message>
date range sanity checks now pass
</commit_message>
<xml_diff>
--- a/tests/data/date_sanity/too_far_back.xlsx
+++ b/tests/data/date_sanity/too_far_back.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/date_sanity/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AABC247F-C1F9-C243-9DFB-55F2CB139A2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E24C8C4-AB00-BB47-A512-A75C16724699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5580" yWindow="2380" windowWidth="23220" windowHeight="13820" xr2:uid="{CF832894-C125-3F4D-A77C-5BE11EEA6BB8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>patient</t>
   </si>
@@ -63,9 +63,6 @@
   </si>
   <si>
     <t>yukf34</t>
-  </si>
-  <si>
-    <t>5/2/1007</t>
   </si>
 </sst>
 </file>
@@ -107,9 +104,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -446,12 +444,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADAB7794-E4FB-6746-A8E0-4C186BFF7A3C}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="10.83203125" style="2"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -475,8 +476,8 @@
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>8</v>
+      <c r="B4" s="1">
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="17" x14ac:dyDescent="0.2">

</xml_diff>